<commit_message>
feat: update Python script for weekly R5 portfolio performance analysis, enhancing evaluation horizon flexibility and improving data loading methods for US and China markets; add new Excel output files reflecting changes
</commit_message>
<xml_diff>
--- a/outputs/analysis_results/01_short-horizon portfolio performance/01_portfolio_weekly_h1_us.xlsx
+++ b/outputs/analysis_results/01_short-horizon portfolio performance/01_portfolio_weekly_h1_us.xlsx
@@ -417,7 +417,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B9"/>
+  <dimension ref="A1:B11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -476,7 +476,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Weekly R5 portfolio summary from step-04 CNN all_h1.xlsx and step-05 benchmark h1.xlsx.</t>
+          <t>Weekly R5 portfolio summary from step-04 CNN all_h{k}.xlsx and step-05 benchmark h{k}.xlsx.</t>
         </is>
       </c>
     </row>
@@ -512,7 +512,7 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Turnover row: Turnover (annualized) on H-L (DH) portfolio.</t>
+          <t>H-L: eval horizon H1 (signal at t, return over 1st future rebalance period).</t>
         </is>
       </c>
     </row>
@@ -524,7 +524,31 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>H-L return stars use Newey-West t-stat on the long-short spread.</t>
+          <t>DH Ret2 / DH Ret3: H-L (DH) annualized return at eval horizons H2 / H3 (2nd / 3rd future rebalance period).</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>note</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>Turnover row: monthly turnover on H-L (DH), paper Table I / GKX (2020) convention (R5 one-week holding ≈ 0.25 month; scaled from backtest Turnover (annualized)).</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>note</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>H-L and DH Ret2/Ret3 return stars use Newey-West t-stat on the long-short spread.</t>
         </is>
       </c>
     </row>
@@ -539,7 +563,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P25"/>
+  <dimension ref="A1:P29"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1534,48 +1558,48 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Turnover</t>
+          <t>DH Ret2</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>90%</t>
+          <t>0.05*** (2.87)</t>
         </is>
       </c>
       <c r="D13" t="inlineStr"/>
       <c r="E13" t="inlineStr">
         <is>
-          <t>88%</t>
+          <t>0.09*** (4.82)</t>
         </is>
       </c>
       <c r="F13" t="inlineStr"/>
       <c r="G13" t="inlineStr">
         <is>
-          <t>77%</t>
+          <t>0.12*** (3.90)</t>
         </is>
       </c>
       <c r="H13" t="inlineStr"/>
       <c r="I13" t="inlineStr">
         <is>
-          <t>13%</t>
+          <t>0.02 (0.24)</t>
         </is>
       </c>
       <c r="J13" t="inlineStr"/>
       <c r="K13" t="inlineStr">
         <is>
-          <t>42%</t>
+          <t>0.10* (1.90)</t>
         </is>
       </c>
       <c r="L13" t="inlineStr"/>
       <c r="M13" t="inlineStr">
         <is>
-          <t>84%</t>
+          <t>0.08** (2.30)</t>
         </is>
       </c>
       <c r="N13" t="inlineStr"/>
       <c r="O13" t="inlineStr">
         <is>
-          <t>62%</t>
+          <t>0.05 (1.04)</t>
         </is>
       </c>
       <c r="P13" t="inlineStr"/>
@@ -1583,166 +1607,110 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>TotalCap-Weight</t>
+          <t>Equal-Weight</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Low</t>
+          <t>DH Ret3</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>-0.03</t>
-        </is>
-      </c>
-      <c r="D14" t="inlineStr">
-        <is>
-          <t>-0.17</t>
-        </is>
-      </c>
+          <t>0.05** (2.46)</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr"/>
       <c r="E14" t="inlineStr">
         <is>
-          <t>-0.03</t>
-        </is>
-      </c>
-      <c r="F14" t="inlineStr">
-        <is>
-          <t>-0.16</t>
-        </is>
-      </c>
+          <t>0.07*** (3.42)</t>
+        </is>
+      </c>
+      <c r="F14" t="inlineStr"/>
       <c r="G14" t="inlineStr">
         <is>
-          <t>-0.02</t>
-        </is>
-      </c>
-      <c r="H14" t="inlineStr">
-        <is>
-          <t>-0.08</t>
-        </is>
-      </c>
+          <t>0.11*** (3.63)</t>
+        </is>
+      </c>
+      <c r="H14" t="inlineStr"/>
       <c r="I14" t="inlineStr">
         <is>
-          <t>0.03</t>
-        </is>
-      </c>
-      <c r="J14" t="inlineStr">
-        <is>
-          <t>0.08</t>
-        </is>
-      </c>
+          <t>0.03 (0.35)</t>
+        </is>
+      </c>
+      <c r="J14" t="inlineStr"/>
       <c r="K14" t="inlineStr">
         <is>
-          <t>0.03</t>
-        </is>
-      </c>
-      <c r="L14" t="inlineStr">
-        <is>
-          <t>0.12</t>
-        </is>
-      </c>
+          <t>0.07 (1.52)</t>
+        </is>
+      </c>
+      <c r="L14" t="inlineStr"/>
       <c r="M14" t="inlineStr">
         <is>
-          <t>-0.04</t>
-        </is>
-      </c>
-      <c r="N14" t="inlineStr">
-        <is>
-          <t>-0.20</t>
-        </is>
-      </c>
+          <t>0.06* (1.75)</t>
+        </is>
+      </c>
+      <c r="N14" t="inlineStr"/>
       <c r="O14" t="inlineStr">
         <is>
-          <t>0.03</t>
-        </is>
-      </c>
-      <c r="P14" t="inlineStr">
-        <is>
-          <t>0.11</t>
-        </is>
-      </c>
+          <t>0.04 (0.71)</t>
+        </is>
+      </c>
+      <c r="P14" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>TotalCap-Weight</t>
+          <t>Equal-Weight</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>Turnover</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>-0.00</t>
-        </is>
-      </c>
-      <c r="D15" t="inlineStr">
-        <is>
-          <t>-0.01</t>
-        </is>
-      </c>
+          <t>696%</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr"/>
       <c r="E15" t="inlineStr">
         <is>
-          <t>0.03</t>
-        </is>
-      </c>
-      <c r="F15" t="inlineStr">
-        <is>
-          <t>0.16</t>
-        </is>
-      </c>
+          <t>674%</t>
+        </is>
+      </c>
+      <c r="F15" t="inlineStr"/>
       <c r="G15" t="inlineStr">
         <is>
-          <t>0.03</t>
-        </is>
-      </c>
-      <c r="H15" t="inlineStr">
-        <is>
-          <t>0.17</t>
-        </is>
-      </c>
+          <t>592%</t>
+        </is>
+      </c>
+      <c r="H15" t="inlineStr"/>
       <c r="I15" t="inlineStr">
         <is>
-          <t>0.05</t>
-        </is>
-      </c>
-      <c r="J15" t="inlineStr">
-        <is>
-          <t>0.17</t>
-        </is>
-      </c>
+          <t>100%</t>
+        </is>
+      </c>
+      <c r="J15" t="inlineStr"/>
       <c r="K15" t="inlineStr">
         <is>
-          <t>0.04</t>
-        </is>
-      </c>
-      <c r="L15" t="inlineStr">
-        <is>
-          <t>0.20</t>
-        </is>
-      </c>
+          <t>326%</t>
+        </is>
+      </c>
+      <c r="L15" t="inlineStr"/>
       <c r="M15" t="inlineStr">
         <is>
-          <t>0.01</t>
-        </is>
-      </c>
-      <c r="N15" t="inlineStr">
-        <is>
-          <t>0.06</t>
-        </is>
-      </c>
+          <t>649%</t>
+        </is>
+      </c>
+      <c r="N15" t="inlineStr"/>
       <c r="O15" t="inlineStr">
         <is>
-          <t>0.04</t>
-        </is>
-      </c>
-      <c r="P15" t="inlineStr">
-        <is>
-          <t>0.21</t>
-        </is>
-      </c>
+          <t>479%</t>
+        </is>
+      </c>
+      <c r="P15" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -1752,77 +1720,77 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>Low</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>0.02</t>
+          <t>-0.03</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
+          <t>-0.17</t>
+        </is>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>-0.03</t>
+        </is>
+      </c>
+      <c r="F16" t="inlineStr">
+        <is>
+          <t>-0.16</t>
+        </is>
+      </c>
+      <c r="G16" t="inlineStr">
+        <is>
+          <t>-0.02</t>
+        </is>
+      </c>
+      <c r="H16" t="inlineStr">
+        <is>
+          <t>-0.08</t>
+        </is>
+      </c>
+      <c r="I16" t="inlineStr">
+        <is>
+          <t>0.03</t>
+        </is>
+      </c>
+      <c r="J16" t="inlineStr">
+        <is>
+          <t>0.08</t>
+        </is>
+      </c>
+      <c r="K16" t="inlineStr">
+        <is>
+          <t>0.03</t>
+        </is>
+      </c>
+      <c r="L16" t="inlineStr">
+        <is>
           <t>0.12</t>
         </is>
       </c>
-      <c r="E16" t="inlineStr">
+      <c r="M16" t="inlineStr">
+        <is>
+          <t>-0.04</t>
+        </is>
+      </c>
+      <c r="N16" t="inlineStr">
+        <is>
+          <t>-0.20</t>
+        </is>
+      </c>
+      <c r="O16" t="inlineStr">
         <is>
           <t>0.03</t>
         </is>
       </c>
-      <c r="F16" t="inlineStr">
-        <is>
-          <t>0.19</t>
-        </is>
-      </c>
-      <c r="G16" t="inlineStr">
-        <is>
-          <t>0.05</t>
-        </is>
-      </c>
-      <c r="H16" t="inlineStr">
-        <is>
-          <t>0.28</t>
-        </is>
-      </c>
-      <c r="I16" t="inlineStr">
-        <is>
-          <t>0.07</t>
-        </is>
-      </c>
-      <c r="J16" t="inlineStr">
-        <is>
-          <t>0.29</t>
-        </is>
-      </c>
-      <c r="K16" t="inlineStr">
-        <is>
-          <t>0.07</t>
-        </is>
-      </c>
-      <c r="L16" t="inlineStr">
-        <is>
-          <t>0.39</t>
-        </is>
-      </c>
-      <c r="M16" t="inlineStr">
-        <is>
-          <t>0.06</t>
-        </is>
-      </c>
-      <c r="N16" t="inlineStr">
-        <is>
-          <t>0.34</t>
-        </is>
-      </c>
-      <c r="O16" t="inlineStr">
-        <is>
-          <t>0.05</t>
-        </is>
-      </c>
       <c r="P16" t="inlineStr">
         <is>
-          <t>0.30</t>
+          <t>0.11</t>
         </is>
       </c>
     </row>
@@ -1834,77 +1802,77 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>2</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
+          <t>-0.00</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>-0.01</t>
+        </is>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>0.03</t>
+        </is>
+      </c>
+      <c r="F17" t="inlineStr">
+        <is>
+          <t>0.16</t>
+        </is>
+      </c>
+      <c r="G17" t="inlineStr">
+        <is>
+          <t>0.03</t>
+        </is>
+      </c>
+      <c r="H17" t="inlineStr">
+        <is>
+          <t>0.17</t>
+        </is>
+      </c>
+      <c r="I17" t="inlineStr">
+        <is>
           <t>0.05</t>
         </is>
       </c>
-      <c r="D17" t="inlineStr">
-        <is>
-          <t>0.31</t>
-        </is>
-      </c>
-      <c r="E17" t="inlineStr">
-        <is>
-          <t>0.05</t>
-        </is>
-      </c>
-      <c r="F17" t="inlineStr">
-        <is>
-          <t>0.29</t>
-        </is>
-      </c>
-      <c r="G17" t="inlineStr">
+      <c r="J17" t="inlineStr">
+        <is>
+          <t>0.17</t>
+        </is>
+      </c>
+      <c r="K17" t="inlineStr">
+        <is>
+          <t>0.04</t>
+        </is>
+      </c>
+      <c r="L17" t="inlineStr">
+        <is>
+          <t>0.20</t>
+        </is>
+      </c>
+      <c r="M17" t="inlineStr">
+        <is>
+          <t>0.01</t>
+        </is>
+      </c>
+      <c r="N17" t="inlineStr">
         <is>
           <t>0.06</t>
         </is>
       </c>
-      <c r="H17" t="inlineStr">
-        <is>
-          <t>0.30</t>
-        </is>
-      </c>
-      <c r="I17" t="inlineStr">
-        <is>
-          <t>0.08</t>
-        </is>
-      </c>
-      <c r="J17" t="inlineStr">
-        <is>
-          <t>0.38</t>
-        </is>
-      </c>
-      <c r="K17" t="inlineStr">
-        <is>
-          <t>0.07</t>
-        </is>
-      </c>
-      <c r="L17" t="inlineStr">
-        <is>
-          <t>0.45</t>
-        </is>
-      </c>
-      <c r="M17" t="inlineStr">
-        <is>
-          <t>0.05</t>
-        </is>
-      </c>
-      <c r="N17" t="inlineStr">
-        <is>
-          <t>0.32</t>
-        </is>
-      </c>
       <c r="O17" t="inlineStr">
         <is>
-          <t>0.06</t>
+          <t>0.04</t>
         </is>
       </c>
       <c r="P17" t="inlineStr">
         <is>
-          <t>0.34</t>
+          <t>0.21</t>
         </is>
       </c>
     </row>
@@ -1916,77 +1884,77 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>3</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
+          <t>0.02</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>0.12</t>
+        </is>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>0.03</t>
+        </is>
+      </c>
+      <c r="F18" t="inlineStr">
+        <is>
+          <t>0.19</t>
+        </is>
+      </c>
+      <c r="G18" t="inlineStr">
+        <is>
+          <t>0.05</t>
+        </is>
+      </c>
+      <c r="H18" t="inlineStr">
+        <is>
+          <t>0.28</t>
+        </is>
+      </c>
+      <c r="I18" t="inlineStr">
+        <is>
           <t>0.07</t>
         </is>
       </c>
-      <c r="D18" t="inlineStr">
-        <is>
-          <t>0.38</t>
-        </is>
-      </c>
-      <c r="E18" t="inlineStr">
+      <c r="J18" t="inlineStr">
+        <is>
+          <t>0.29</t>
+        </is>
+      </c>
+      <c r="K18" t="inlineStr">
+        <is>
+          <t>0.07</t>
+        </is>
+      </c>
+      <c r="L18" t="inlineStr">
+        <is>
+          <t>0.39</t>
+        </is>
+      </c>
+      <c r="M18" t="inlineStr">
         <is>
           <t>0.06</t>
         </is>
       </c>
-      <c r="F18" t="inlineStr">
+      <c r="N18" t="inlineStr">
         <is>
           <t>0.34</t>
         </is>
       </c>
-      <c r="G18" t="inlineStr">
-        <is>
-          <t>0.07</t>
-        </is>
-      </c>
-      <c r="H18" t="inlineStr">
-        <is>
-          <t>0.39</t>
-        </is>
-      </c>
-      <c r="I18" t="inlineStr">
-        <is>
-          <t>0.09</t>
-        </is>
-      </c>
-      <c r="J18" t="inlineStr">
-        <is>
-          <t>0.47</t>
-        </is>
-      </c>
-      <c r="K18" t="inlineStr">
-        <is>
-          <t>0.10</t>
-        </is>
-      </c>
-      <c r="L18" t="inlineStr">
-        <is>
-          <t>0.59</t>
-        </is>
-      </c>
-      <c r="M18" t="inlineStr">
-        <is>
-          <t>0.07</t>
-        </is>
-      </c>
-      <c r="N18" t="inlineStr">
-        <is>
-          <t>0.45</t>
-        </is>
-      </c>
       <c r="O18" t="inlineStr">
         <is>
-          <t>0.08</t>
+          <t>0.05</t>
         </is>
       </c>
       <c r="P18" t="inlineStr">
         <is>
-          <t>0.49</t>
+          <t>0.30</t>
         </is>
       </c>
     </row>
@@ -1998,77 +1966,77 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>4</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
+          <t>0.05</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>0.31</t>
+        </is>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>0.05</t>
+        </is>
+      </c>
+      <c r="F19" t="inlineStr">
+        <is>
+          <t>0.29</t>
+        </is>
+      </c>
+      <c r="G19" t="inlineStr">
+        <is>
+          <t>0.06</t>
+        </is>
+      </c>
+      <c r="H19" t="inlineStr">
+        <is>
+          <t>0.30</t>
+        </is>
+      </c>
+      <c r="I19" t="inlineStr">
+        <is>
           <t>0.08</t>
         </is>
       </c>
-      <c r="D19" t="inlineStr">
-        <is>
-          <t>0.47</t>
-        </is>
-      </c>
-      <c r="E19" t="inlineStr">
-        <is>
-          <t>0.09</t>
-        </is>
-      </c>
-      <c r="F19" t="inlineStr">
-        <is>
-          <t>0.49</t>
-        </is>
-      </c>
-      <c r="G19" t="inlineStr">
+      <c r="J19" t="inlineStr">
+        <is>
+          <t>0.38</t>
+        </is>
+      </c>
+      <c r="K19" t="inlineStr">
         <is>
           <t>0.07</t>
         </is>
       </c>
-      <c r="H19" t="inlineStr">
-        <is>
-          <t>0.40</t>
-        </is>
-      </c>
-      <c r="I19" t="inlineStr">
-        <is>
-          <t>0.09</t>
-        </is>
-      </c>
-      <c r="J19" t="inlineStr">
-        <is>
-          <t>0.55</t>
-        </is>
-      </c>
-      <c r="K19" t="inlineStr">
-        <is>
-          <t>0.09</t>
-        </is>
-      </c>
       <c r="L19" t="inlineStr">
         <is>
-          <t>0.54</t>
+          <t>0.45</t>
         </is>
       </c>
       <c r="M19" t="inlineStr">
         <is>
-          <t>0.10</t>
+          <t>0.05</t>
         </is>
       </c>
       <c r="N19" t="inlineStr">
         <is>
-          <t>0.59</t>
+          <t>0.32</t>
         </is>
       </c>
       <c r="O19" t="inlineStr">
         <is>
-          <t>0.09</t>
+          <t>0.06</t>
         </is>
       </c>
       <c r="P19" t="inlineStr">
         <is>
-          <t>0.56</t>
+          <t>0.34</t>
         </is>
       </c>
     </row>
@@ -2080,77 +2048,77 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>5</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
+          <t>0.07</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>0.38</t>
+        </is>
+      </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>0.06</t>
+        </is>
+      </c>
+      <c r="F20" t="inlineStr">
+        <is>
+          <t>0.34</t>
+        </is>
+      </c>
+      <c r="G20" t="inlineStr">
+        <is>
+          <t>0.07</t>
+        </is>
+      </c>
+      <c r="H20" t="inlineStr">
+        <is>
+          <t>0.39</t>
+        </is>
+      </c>
+      <c r="I20" t="inlineStr">
+        <is>
+          <t>0.09</t>
+        </is>
+      </c>
+      <c r="J20" t="inlineStr">
+        <is>
+          <t>0.47</t>
+        </is>
+      </c>
+      <c r="K20" t="inlineStr">
+        <is>
           <t>0.10</t>
         </is>
       </c>
-      <c r="D20" t="inlineStr">
-        <is>
-          <t>0.54</t>
-        </is>
-      </c>
-      <c r="E20" t="inlineStr">
-        <is>
-          <t>0.09</t>
-        </is>
-      </c>
-      <c r="F20" t="inlineStr">
-        <is>
-          <t>0.52</t>
-        </is>
-      </c>
-      <c r="G20" t="inlineStr">
+      <c r="L20" t="inlineStr">
+        <is>
+          <t>0.59</t>
+        </is>
+      </c>
+      <c r="M20" t="inlineStr">
+        <is>
+          <t>0.07</t>
+        </is>
+      </c>
+      <c r="N20" t="inlineStr">
+        <is>
+          <t>0.45</t>
+        </is>
+      </c>
+      <c r="O20" t="inlineStr">
         <is>
           <t>0.08</t>
         </is>
       </c>
-      <c r="H20" t="inlineStr">
-        <is>
-          <t>0.47</t>
-        </is>
-      </c>
-      <c r="I20" t="inlineStr">
-        <is>
-          <t>0.09</t>
-        </is>
-      </c>
-      <c r="J20" t="inlineStr">
-        <is>
-          <t>0.58</t>
-        </is>
-      </c>
-      <c r="K20" t="inlineStr">
-        <is>
-          <t>0.09</t>
-        </is>
-      </c>
-      <c r="L20" t="inlineStr">
-        <is>
-          <t>0.51</t>
-        </is>
-      </c>
-      <c r="M20" t="inlineStr">
-        <is>
-          <t>0.11</t>
-        </is>
-      </c>
-      <c r="N20" t="inlineStr">
-        <is>
-          <t>0.62</t>
-        </is>
-      </c>
-      <c r="O20" t="inlineStr">
-        <is>
-          <t>0.11</t>
-        </is>
-      </c>
       <c r="P20" t="inlineStr">
         <is>
-          <t>0.59</t>
+          <t>0.49</t>
         </is>
       </c>
     </row>
@@ -2162,77 +2130,77 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>6</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>0.13</t>
+          <t>0.08</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>0.71</t>
+          <t>0.47</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
         <is>
+          <t>0.09</t>
+        </is>
+      </c>
+      <c r="F21" t="inlineStr">
+        <is>
+          <t>0.49</t>
+        </is>
+      </c>
+      <c r="G21" t="inlineStr">
+        <is>
+          <t>0.07</t>
+        </is>
+      </c>
+      <c r="H21" t="inlineStr">
+        <is>
+          <t>0.40</t>
+        </is>
+      </c>
+      <c r="I21" t="inlineStr">
+        <is>
+          <t>0.09</t>
+        </is>
+      </c>
+      <c r="J21" t="inlineStr">
+        <is>
+          <t>0.55</t>
+        </is>
+      </c>
+      <c r="K21" t="inlineStr">
+        <is>
+          <t>0.09</t>
+        </is>
+      </c>
+      <c r="L21" t="inlineStr">
+        <is>
+          <t>0.54</t>
+        </is>
+      </c>
+      <c r="M21" t="inlineStr">
+        <is>
           <t>0.10</t>
         </is>
       </c>
-      <c r="F21" t="inlineStr">
+      <c r="N21" t="inlineStr">
+        <is>
+          <t>0.59</t>
+        </is>
+      </c>
+      <c r="O21" t="inlineStr">
+        <is>
+          <t>0.09</t>
+        </is>
+      </c>
+      <c r="P21" t="inlineStr">
         <is>
           <t>0.56</t>
-        </is>
-      </c>
-      <c r="G21" t="inlineStr">
-        <is>
-          <t>0.08</t>
-        </is>
-      </c>
-      <c r="H21" t="inlineStr">
-        <is>
-          <t>0.46</t>
-        </is>
-      </c>
-      <c r="I21" t="inlineStr">
-        <is>
-          <t>0.09</t>
-        </is>
-      </c>
-      <c r="J21" t="inlineStr">
-        <is>
-          <t>0.57</t>
-        </is>
-      </c>
-      <c r="K21" t="inlineStr">
-        <is>
-          <t>0.12</t>
-        </is>
-      </c>
-      <c r="L21" t="inlineStr">
-        <is>
-          <t>0.58</t>
-        </is>
-      </c>
-      <c r="M21" t="inlineStr">
-        <is>
-          <t>0.14</t>
-        </is>
-      </c>
-      <c r="N21" t="inlineStr">
-        <is>
-          <t>0.73</t>
-        </is>
-      </c>
-      <c r="O21" t="inlineStr">
-        <is>
-          <t>0.11</t>
-        </is>
-      </c>
-      <c r="P21" t="inlineStr">
-        <is>
-          <t>0.58</t>
         </is>
       </c>
     </row>
@@ -2244,77 +2212,77 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>7</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>0.15</t>
+          <t>0.10</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>0.78</t>
+          <t>0.54</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
         <is>
+          <t>0.09</t>
+        </is>
+      </c>
+      <c r="F22" t="inlineStr">
+        <is>
+          <t>0.52</t>
+        </is>
+      </c>
+      <c r="G22" t="inlineStr">
+        <is>
+          <t>0.08</t>
+        </is>
+      </c>
+      <c r="H22" t="inlineStr">
+        <is>
+          <t>0.47</t>
+        </is>
+      </c>
+      <c r="I22" t="inlineStr">
+        <is>
+          <t>0.09</t>
+        </is>
+      </c>
+      <c r="J22" t="inlineStr">
+        <is>
+          <t>0.58</t>
+        </is>
+      </c>
+      <c r="K22" t="inlineStr">
+        <is>
+          <t>0.09</t>
+        </is>
+      </c>
+      <c r="L22" t="inlineStr">
+        <is>
+          <t>0.51</t>
+        </is>
+      </c>
+      <c r="M22" t="inlineStr">
+        <is>
           <t>0.11</t>
         </is>
       </c>
-      <c r="F22" t="inlineStr">
+      <c r="N22" t="inlineStr">
+        <is>
+          <t>0.62</t>
+        </is>
+      </c>
+      <c r="O22" t="inlineStr">
+        <is>
+          <t>0.11</t>
+        </is>
+      </c>
+      <c r="P22" t="inlineStr">
         <is>
           <t>0.59</t>
-        </is>
-      </c>
-      <c r="G22" t="inlineStr">
-        <is>
-          <t>0.10</t>
-        </is>
-      </c>
-      <c r="H22" t="inlineStr">
-        <is>
-          <t>0.55</t>
-        </is>
-      </c>
-      <c r="I22" t="inlineStr">
-        <is>
-          <t>0.10</t>
-        </is>
-      </c>
-      <c r="J22" t="inlineStr">
-        <is>
-          <t>0.55</t>
-        </is>
-      </c>
-      <c r="K22" t="inlineStr">
-        <is>
-          <t>0.12</t>
-        </is>
-      </c>
-      <c r="L22" t="inlineStr">
-        <is>
-          <t>0.48</t>
-        </is>
-      </c>
-      <c r="M22" t="inlineStr">
-        <is>
-          <t>0.17</t>
-        </is>
-      </c>
-      <c r="N22" t="inlineStr">
-        <is>
-          <t>0.72</t>
-        </is>
-      </c>
-      <c r="O22" t="inlineStr">
-        <is>
-          <t>0.12</t>
-        </is>
-      </c>
-      <c r="P22" t="inlineStr">
-        <is>
-          <t>0.49</t>
         </is>
       </c>
     </row>
@@ -2326,37 +2294,37 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>8</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>0.19</t>
+          <t>0.13</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>0.93</t>
+          <t>0.71</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>0.15</t>
+          <t>0.10</t>
         </is>
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>0.80</t>
+          <t>0.56</t>
         </is>
       </c>
       <c r="G23" t="inlineStr">
         <is>
-          <t>0.13</t>
+          <t>0.08</t>
         </is>
       </c>
       <c r="H23" t="inlineStr">
         <is>
-          <t>0.76</t>
+          <t>0.46</t>
         </is>
       </c>
       <c r="I23" t="inlineStr">
@@ -2366,27 +2334,27 @@
       </c>
       <c r="J23" t="inlineStr">
         <is>
-          <t>0.42</t>
+          <t>0.57</t>
         </is>
       </c>
       <c r="K23" t="inlineStr">
         <is>
+          <t>0.12</t>
+        </is>
+      </c>
+      <c r="L23" t="inlineStr">
+        <is>
+          <t>0.58</t>
+        </is>
+      </c>
+      <c r="M23" t="inlineStr">
+        <is>
           <t>0.14</t>
         </is>
       </c>
-      <c r="L23" t="inlineStr">
-        <is>
-          <t>0.40</t>
-        </is>
-      </c>
-      <c r="M23" t="inlineStr">
-        <is>
-          <t>0.16</t>
-        </is>
-      </c>
       <c r="N23" t="inlineStr">
         <is>
-          <t>0.53</t>
+          <t>0.73</t>
         </is>
       </c>
       <c r="O23" t="inlineStr">
@@ -2396,7 +2364,7 @@
       </c>
       <c r="P23" t="inlineStr">
         <is>
-          <t>0.34</t>
+          <t>0.58</t>
         </is>
       </c>
     </row>
@@ -2408,77 +2376,77 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>H-L</t>
+          <t>9</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>0.22*** (6.17)</t>
+          <t>0.15</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>1.52</t>
+          <t>0.78</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>0.18*** (5.87)</t>
+          <t>0.11</t>
         </is>
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>1.50</t>
+          <t>0.59</t>
         </is>
       </c>
       <c r="G24" t="inlineStr">
         <is>
-          <t>0.15*** (4.45)</t>
+          <t>0.10</t>
         </is>
       </c>
       <c r="H24" t="inlineStr">
         <is>
-          <t>1.23</t>
+          <t>0.55</t>
         </is>
       </c>
       <c r="I24" t="inlineStr">
         <is>
-          <t>0.06 (0.67)</t>
+          <t>0.10</t>
         </is>
       </c>
       <c r="J24" t="inlineStr">
         <is>
+          <t>0.55</t>
+        </is>
+      </c>
+      <c r="K24" t="inlineStr">
+        <is>
+          <t>0.12</t>
+        </is>
+      </c>
+      <c r="L24" t="inlineStr">
+        <is>
+          <t>0.48</t>
+        </is>
+      </c>
+      <c r="M24" t="inlineStr">
+        <is>
           <t>0.17</t>
         </is>
       </c>
-      <c r="K24" t="inlineStr">
-        <is>
-          <t>0.11* (1.82)</t>
-        </is>
-      </c>
-      <c r="L24" t="inlineStr">
-        <is>
-          <t>0.41</t>
-        </is>
-      </c>
-      <c r="M24" t="inlineStr">
-        <is>
-          <t>0.20*** (3.94)</t>
-        </is>
-      </c>
       <c r="N24" t="inlineStr">
         <is>
-          <t>0.89</t>
+          <t>0.72</t>
         </is>
       </c>
       <c r="O24" t="inlineStr">
         <is>
-          <t>0.08 (1.55)</t>
+          <t>0.12</t>
         </is>
       </c>
       <c r="P24" t="inlineStr">
         <is>
-          <t>0.35</t>
+          <t>0.49</t>
         </is>
       </c>
     </row>
@@ -2490,51 +2458,323 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>0.19</t>
+        </is>
+      </c>
+      <c r="D25" t="inlineStr">
+        <is>
+          <t>0.93</t>
+        </is>
+      </c>
+      <c r="E25" t="inlineStr">
+        <is>
+          <t>0.15</t>
+        </is>
+      </c>
+      <c r="F25" t="inlineStr">
+        <is>
+          <t>0.80</t>
+        </is>
+      </c>
+      <c r="G25" t="inlineStr">
+        <is>
+          <t>0.13</t>
+        </is>
+      </c>
+      <c r="H25" t="inlineStr">
+        <is>
+          <t>0.76</t>
+        </is>
+      </c>
+      <c r="I25" t="inlineStr">
+        <is>
+          <t>0.09</t>
+        </is>
+      </c>
+      <c r="J25" t="inlineStr">
+        <is>
+          <t>0.42</t>
+        </is>
+      </c>
+      <c r="K25" t="inlineStr">
+        <is>
+          <t>0.14</t>
+        </is>
+      </c>
+      <c r="L25" t="inlineStr">
+        <is>
+          <t>0.40</t>
+        </is>
+      </c>
+      <c r="M25" t="inlineStr">
+        <is>
+          <t>0.16</t>
+        </is>
+      </c>
+      <c r="N25" t="inlineStr">
+        <is>
+          <t>0.53</t>
+        </is>
+      </c>
+      <c r="O25" t="inlineStr">
+        <is>
+          <t>0.11</t>
+        </is>
+      </c>
+      <c r="P25" t="inlineStr">
+        <is>
+          <t>0.34</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>TotalCap-Weight</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>H-L</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>0.22*** (6.17)</t>
+        </is>
+      </c>
+      <c r="D26" t="inlineStr">
+        <is>
+          <t>1.52</t>
+        </is>
+      </c>
+      <c r="E26" t="inlineStr">
+        <is>
+          <t>0.18*** (5.87)</t>
+        </is>
+      </c>
+      <c r="F26" t="inlineStr">
+        <is>
+          <t>1.50</t>
+        </is>
+      </c>
+      <c r="G26" t="inlineStr">
+        <is>
+          <t>0.15*** (4.45)</t>
+        </is>
+      </c>
+      <c r="H26" t="inlineStr">
+        <is>
+          <t>1.23</t>
+        </is>
+      </c>
+      <c r="I26" t="inlineStr">
+        <is>
+          <t>0.06 (0.67)</t>
+        </is>
+      </c>
+      <c r="J26" t="inlineStr">
+        <is>
+          <t>0.17</t>
+        </is>
+      </c>
+      <c r="K26" t="inlineStr">
+        <is>
+          <t>0.11* (1.82)</t>
+        </is>
+      </c>
+      <c r="L26" t="inlineStr">
+        <is>
+          <t>0.41</t>
+        </is>
+      </c>
+      <c r="M26" t="inlineStr">
+        <is>
+          <t>0.20*** (3.94)</t>
+        </is>
+      </c>
+      <c r="N26" t="inlineStr">
+        <is>
+          <t>0.89</t>
+        </is>
+      </c>
+      <c r="O26" t="inlineStr">
+        <is>
+          <t>0.08 (1.55)</t>
+        </is>
+      </c>
+      <c r="P26" t="inlineStr">
+        <is>
+          <t>0.35</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>TotalCap-Weight</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>DH Ret2</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>0.00 (0.19)</t>
+        </is>
+      </c>
+      <c r="D27" t="inlineStr"/>
+      <c r="E27" t="inlineStr">
+        <is>
+          <t>0.01 (0.21)</t>
+        </is>
+      </c>
+      <c r="F27" t="inlineStr"/>
+      <c r="G27" t="inlineStr">
+        <is>
+          <t>0.02 (0.70)</t>
+        </is>
+      </c>
+      <c r="H27" t="inlineStr"/>
+      <c r="I27" t="inlineStr">
+        <is>
+          <t>0.05 (0.56)</t>
+        </is>
+      </c>
+      <c r="J27" t="inlineStr"/>
+      <c r="K27" t="inlineStr">
+        <is>
+          <t>0.01 (0.19)</t>
+        </is>
+      </c>
+      <c r="L27" t="inlineStr"/>
+      <c r="M27" t="inlineStr">
+        <is>
+          <t>0.02 (0.43)</t>
+        </is>
+      </c>
+      <c r="N27" t="inlineStr"/>
+      <c r="O27" t="inlineStr">
+        <is>
+          <t>0.02 (0.46)</t>
+        </is>
+      </c>
+      <c r="P27" t="inlineStr"/>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>TotalCap-Weight</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>DH Ret3</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>0.02 (0.69)</t>
+        </is>
+      </c>
+      <c r="D28" t="inlineStr"/>
+      <c r="E28" t="inlineStr">
+        <is>
+          <t>-0.01 (-0.31)</t>
+        </is>
+      </c>
+      <c r="F28" t="inlineStr"/>
+      <c r="G28" t="inlineStr">
+        <is>
+          <t>0.01 (0.54)</t>
+        </is>
+      </c>
+      <c r="H28" t="inlineStr"/>
+      <c r="I28" t="inlineStr">
+        <is>
+          <t>0.05 (0.52)</t>
+        </is>
+      </c>
+      <c r="J28" t="inlineStr"/>
+      <c r="K28" t="inlineStr">
+        <is>
+          <t>-0.01 (-0.16)</t>
+        </is>
+      </c>
+      <c r="L28" t="inlineStr"/>
+      <c r="M28" t="inlineStr">
+        <is>
+          <t>-0.00 (-0.11)</t>
+        </is>
+      </c>
+      <c r="N28" t="inlineStr"/>
+      <c r="O28" t="inlineStr">
+        <is>
+          <t>0.06 (0.87)</t>
+        </is>
+      </c>
+      <c r="P28" t="inlineStr"/>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>TotalCap-Weight</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
           <t>Turnover</t>
         </is>
       </c>
-      <c r="C25" t="inlineStr">
-        <is>
-          <t>98%</t>
-        </is>
-      </c>
-      <c r="D25" t="inlineStr"/>
-      <c r="E25" t="inlineStr">
-        <is>
-          <t>94%</t>
-        </is>
-      </c>
-      <c r="F25" t="inlineStr"/>
-      <c r="G25" t="inlineStr">
-        <is>
-          <t>84%</t>
-        </is>
-      </c>
-      <c r="H25" t="inlineStr"/>
-      <c r="I25" t="inlineStr">
-        <is>
-          <t>20%</t>
-        </is>
-      </c>
-      <c r="J25" t="inlineStr"/>
-      <c r="K25" t="inlineStr">
-        <is>
-          <t>56%</t>
-        </is>
-      </c>
-      <c r="L25" t="inlineStr"/>
-      <c r="M25" t="inlineStr">
-        <is>
-          <t>95%</t>
-        </is>
-      </c>
-      <c r="N25" t="inlineStr"/>
-      <c r="O25" t="inlineStr">
-        <is>
-          <t>74%</t>
-        </is>
-      </c>
-      <c r="P25" t="inlineStr"/>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>756%</t>
+        </is>
+      </c>
+      <c r="D29" t="inlineStr"/>
+      <c r="E29" t="inlineStr">
+        <is>
+          <t>724%</t>
+        </is>
+      </c>
+      <c r="F29" t="inlineStr"/>
+      <c r="G29" t="inlineStr">
+        <is>
+          <t>646%</t>
+        </is>
+      </c>
+      <c r="H29" t="inlineStr"/>
+      <c r="I29" t="inlineStr">
+        <is>
+          <t>152%</t>
+        </is>
+      </c>
+      <c r="J29" t="inlineStr"/>
+      <c r="K29" t="inlineStr">
+        <is>
+          <t>428%</t>
+        </is>
+      </c>
+      <c r="L29" t="inlineStr"/>
+      <c r="M29" t="inlineStr">
+        <is>
+          <t>731%</t>
+        </is>
+      </c>
+      <c r="N29" t="inlineStr"/>
+      <c r="O29" t="inlineStr">
+        <is>
+          <t>569%</t>
+        </is>
+      </c>
+      <c r="P29" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -2547,7 +2787,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I25"/>
+  <dimension ref="A1:I29"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2968,95 +3208,95 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Turnover</t>
+          <t>DH Ret2</t>
         </is>
       </c>
       <c r="C13" t="n">
-        <v>90.43000000000001</v>
+        <v>0.0536</v>
       </c>
       <c r="D13" t="n">
-        <v>87.58</v>
+        <v>0.09379999999999999</v>
       </c>
       <c r="E13" t="n">
-        <v>76.98</v>
+        <v>0.1244</v>
       </c>
       <c r="F13" t="n">
-        <v>13.02</v>
+        <v>0.0175</v>
       </c>
       <c r="G13" t="n">
-        <v>42.44</v>
+        <v>0.0968</v>
       </c>
       <c r="H13" t="n">
-        <v>84.40000000000001</v>
+        <v>0.0785</v>
       </c>
       <c r="I13" t="n">
-        <v>62.32</v>
+        <v>0.0511</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>TotalCap-Weight</t>
+          <t>Equal-Weight</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Low</t>
+          <t>DH Ret3</t>
         </is>
       </c>
       <c r="C14" t="n">
-        <v>-0.027</v>
+        <v>0.0457</v>
       </c>
       <c r="D14" t="n">
-        <v>-0.0289</v>
+        <v>0.06619999999999999</v>
       </c>
       <c r="E14" t="n">
-        <v>-0.0165</v>
+        <v>0.1101</v>
       </c>
       <c r="F14" t="n">
-        <v>0.0319</v>
+        <v>0.0258</v>
       </c>
       <c r="G14" t="n">
-        <v>0.0269</v>
+        <v>0.07190000000000001</v>
       </c>
       <c r="H14" t="n">
-        <v>-0.045</v>
+        <v>0.06320000000000001</v>
       </c>
       <c r="I14" t="n">
-        <v>0.0261</v>
+        <v>0.0363</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>TotalCap-Weight</t>
+          <t>Equal-Weight</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>Turnover</t>
         </is>
       </c>
       <c r="C15" t="n">
-        <v>-0.0015</v>
+        <v>695.6153846153848</v>
       </c>
       <c r="D15" t="n">
-        <v>0.0291</v>
+        <v>673.6923076923076</v>
       </c>
       <c r="E15" t="n">
-        <v>0.0337</v>
+        <v>592.1538461538462</v>
       </c>
       <c r="F15" t="n">
-        <v>0.0517</v>
+        <v>100.1538461538461</v>
       </c>
       <c r="G15" t="n">
-        <v>0.0357</v>
+        <v>326.4615384615385</v>
       </c>
       <c r="H15" t="n">
-        <v>0.0105</v>
+        <v>649.2307692307693</v>
       </c>
       <c r="I15" t="n">
-        <v>0.0402</v>
+        <v>479.3846153846154</v>
       </c>
     </row>
     <row r="16">
@@ -3067,29 +3307,29 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>Low</t>
         </is>
       </c>
       <c r="C16" t="n">
-        <v>0.0205</v>
+        <v>-0.027</v>
       </c>
       <c r="D16" t="n">
-        <v>0.0339</v>
+        <v>-0.0289</v>
       </c>
       <c r="E16" t="n">
-        <v>0.0547</v>
+        <v>-0.0165</v>
       </c>
       <c r="F16" t="n">
-        <v>0.0732</v>
+        <v>0.0319</v>
       </c>
       <c r="G16" t="n">
-        <v>0.0655</v>
+        <v>0.0269</v>
       </c>
       <c r="H16" t="n">
-        <v>0.0565</v>
+        <v>-0.045</v>
       </c>
       <c r="I16" t="n">
-        <v>0.0521</v>
+        <v>0.0261</v>
       </c>
     </row>
     <row r="17">
@@ -3100,29 +3340,29 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>2</t>
         </is>
       </c>
       <c r="C17" t="n">
-        <v>0.0548</v>
+        <v>-0.0015</v>
       </c>
       <c r="D17" t="n">
-        <v>0.0523</v>
+        <v>0.0291</v>
       </c>
       <c r="E17" t="n">
-        <v>0.0566</v>
+        <v>0.0337</v>
       </c>
       <c r="F17" t="n">
-        <v>0.079</v>
+        <v>0.0517</v>
       </c>
       <c r="G17" t="n">
-        <v>0.0746</v>
+        <v>0.0357</v>
       </c>
       <c r="H17" t="n">
-        <v>0.0537</v>
+        <v>0.0105</v>
       </c>
       <c r="I17" t="n">
-        <v>0.0581</v>
+        <v>0.0402</v>
       </c>
     </row>
     <row r="18">
@@ -3133,29 +3373,29 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>3</t>
         </is>
       </c>
       <c r="C18" t="n">
-        <v>0.0682</v>
+        <v>0.0205</v>
       </c>
       <c r="D18" t="n">
-        <v>0.0624</v>
+        <v>0.0339</v>
       </c>
       <c r="E18" t="n">
-        <v>0.0711</v>
+        <v>0.0547</v>
       </c>
       <c r="F18" t="n">
-        <v>0.0864</v>
+        <v>0.0732</v>
       </c>
       <c r="G18" t="n">
-        <v>0.0979</v>
+        <v>0.0655</v>
       </c>
       <c r="H18" t="n">
-        <v>0.0726</v>
+        <v>0.0565</v>
       </c>
       <c r="I18" t="n">
-        <v>0.0813</v>
+        <v>0.0521</v>
       </c>
     </row>
     <row r="19">
@@ -3166,29 +3406,29 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>4</t>
         </is>
       </c>
       <c r="C19" t="n">
-        <v>0.0847</v>
+        <v>0.0548</v>
       </c>
       <c r="D19" t="n">
-        <v>0.08690000000000001</v>
+        <v>0.0523</v>
       </c>
       <c r="E19" t="n">
-        <v>0.0725</v>
+        <v>0.0566</v>
       </c>
       <c r="F19" t="n">
-        <v>0.09279999999999999</v>
+        <v>0.079</v>
       </c>
       <c r="G19" t="n">
-        <v>0.0946</v>
+        <v>0.0746</v>
       </c>
       <c r="H19" t="n">
-        <v>0.101</v>
+        <v>0.0537</v>
       </c>
       <c r="I19" t="n">
-        <v>0.09379999999999999</v>
+        <v>0.0581</v>
       </c>
     </row>
     <row r="20">
@@ -3199,29 +3439,29 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>5</t>
         </is>
       </c>
       <c r="C20" t="n">
-        <v>0.098</v>
+        <v>0.0682</v>
       </c>
       <c r="D20" t="n">
-        <v>0.09229999999999999</v>
+        <v>0.0624</v>
       </c>
       <c r="E20" t="n">
-        <v>0.082</v>
+        <v>0.0711</v>
       </c>
       <c r="F20" t="n">
-        <v>0.0949</v>
+        <v>0.0864</v>
       </c>
       <c r="G20" t="n">
-        <v>0.0929</v>
+        <v>0.0979</v>
       </c>
       <c r="H20" t="n">
-        <v>0.1111</v>
+        <v>0.0726</v>
       </c>
       <c r="I20" t="n">
-        <v>0.1067</v>
+        <v>0.0813</v>
       </c>
     </row>
     <row r="21">
@@ -3232,29 +3472,29 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>6</t>
         </is>
       </c>
       <c r="C21" t="n">
-        <v>0.132</v>
+        <v>0.0847</v>
       </c>
       <c r="D21" t="n">
-        <v>0.1021</v>
+        <v>0.08690000000000001</v>
       </c>
       <c r="E21" t="n">
-        <v>0.0809</v>
+        <v>0.0725</v>
       </c>
       <c r="F21" t="n">
-        <v>0.09329999999999999</v>
+        <v>0.09279999999999999</v>
       </c>
       <c r="G21" t="n">
-        <v>0.1212</v>
+        <v>0.0946</v>
       </c>
       <c r="H21" t="n">
-        <v>0.1441</v>
+        <v>0.101</v>
       </c>
       <c r="I21" t="n">
-        <v>0.1142</v>
+        <v>0.09379999999999999</v>
       </c>
     </row>
     <row r="22">
@@ -3265,29 +3505,29 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>7</t>
         </is>
       </c>
       <c r="C22" t="n">
-        <v>0.1525</v>
+        <v>0.098</v>
       </c>
       <c r="D22" t="n">
-        <v>0.1084</v>
+        <v>0.09229999999999999</v>
       </c>
       <c r="E22" t="n">
-        <v>0.0953</v>
+        <v>0.082</v>
       </c>
       <c r="F22" t="n">
-        <v>0.095</v>
+        <v>0.0949</v>
       </c>
       <c r="G22" t="n">
-        <v>0.1207</v>
+        <v>0.0929</v>
       </c>
       <c r="H22" t="n">
-        <v>0.1723</v>
+        <v>0.1111</v>
       </c>
       <c r="I22" t="n">
-        <v>0.1173</v>
+        <v>0.1067</v>
       </c>
     </row>
     <row r="23">
@@ -3298,29 +3538,29 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>8</t>
         </is>
       </c>
       <c r="C23" t="n">
-        <v>0.1901</v>
+        <v>0.132</v>
       </c>
       <c r="D23" t="n">
-        <v>0.1502</v>
+        <v>0.1021</v>
       </c>
       <c r="E23" t="n">
-        <v>0.1336</v>
+        <v>0.0809</v>
       </c>
       <c r="F23" t="n">
-        <v>0.0919</v>
+        <v>0.09329999999999999</v>
       </c>
       <c r="G23" t="n">
-        <v>0.1355</v>
+        <v>0.1212</v>
       </c>
       <c r="H23" t="n">
-        <v>0.16</v>
+        <v>0.1441</v>
       </c>
       <c r="I23" t="n">
-        <v>0.1079</v>
+        <v>0.1142</v>
       </c>
     </row>
     <row r="24">
@@ -3331,29 +3571,29 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>H-L</t>
+          <t>9</t>
         </is>
       </c>
       <c r="C24" t="n">
-        <v>0.2171</v>
+        <v>0.1525</v>
       </c>
       <c r="D24" t="n">
-        <v>0.1791</v>
+        <v>0.1084</v>
       </c>
       <c r="E24" t="n">
-        <v>0.1501</v>
+        <v>0.0953</v>
       </c>
       <c r="F24" t="n">
-        <v>0.0601</v>
+        <v>0.095</v>
       </c>
       <c r="G24" t="n">
-        <v>0.1086</v>
+        <v>0.1207</v>
       </c>
       <c r="H24" t="n">
-        <v>0.205</v>
+        <v>0.1723</v>
       </c>
       <c r="I24" t="n">
-        <v>0.0818</v>
+        <v>0.1173</v>
       </c>
     </row>
     <row r="25">
@@ -3364,29 +3604,161 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="C25" t="n">
+        <v>0.1901</v>
+      </c>
+      <c r="D25" t="n">
+        <v>0.1502</v>
+      </c>
+      <c r="E25" t="n">
+        <v>0.1336</v>
+      </c>
+      <c r="F25" t="n">
+        <v>0.0919</v>
+      </c>
+      <c r="G25" t="n">
+        <v>0.1355</v>
+      </c>
+      <c r="H25" t="n">
+        <v>0.16</v>
+      </c>
+      <c r="I25" t="n">
+        <v>0.1079</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>TotalCap-Weight</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>H-L</t>
+        </is>
+      </c>
+      <c r="C26" t="n">
+        <v>0.2171</v>
+      </c>
+      <c r="D26" t="n">
+        <v>0.1791</v>
+      </c>
+      <c r="E26" t="n">
+        <v>0.1501</v>
+      </c>
+      <c r="F26" t="n">
+        <v>0.0601</v>
+      </c>
+      <c r="G26" t="n">
+        <v>0.1086</v>
+      </c>
+      <c r="H26" t="n">
+        <v>0.205</v>
+      </c>
+      <c r="I26" t="n">
+        <v>0.0818</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>TotalCap-Weight</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>DH Ret2</t>
+        </is>
+      </c>
+      <c r="C27" t="n">
+        <v>0.0044</v>
+      </c>
+      <c r="D27" t="n">
+        <v>0.0053</v>
+      </c>
+      <c r="E27" t="n">
+        <v>0.0241</v>
+      </c>
+      <c r="F27" t="n">
+        <v>0.0485</v>
+      </c>
+      <c r="G27" t="n">
+        <v>0.0105</v>
+      </c>
+      <c r="H27" t="n">
+        <v>0.0214</v>
+      </c>
+      <c r="I27" t="n">
+        <v>0.0235</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>TotalCap-Weight</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>DH Ret3</t>
+        </is>
+      </c>
+      <c r="C28" t="n">
+        <v>0.0191</v>
+      </c>
+      <c r="D28" t="n">
+        <v>-0.0075</v>
+      </c>
+      <c r="E28" t="n">
+        <v>0.015</v>
+      </c>
+      <c r="F28" t="n">
+        <v>0.0452</v>
+      </c>
+      <c r="G28" t="n">
+        <v>-0.0081</v>
+      </c>
+      <c r="H28" t="n">
+        <v>-0.0049</v>
+      </c>
+      <c r="I28" t="n">
+        <v>0.0557</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>TotalCap-Weight</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
           <t>Turnover</t>
         </is>
       </c>
-      <c r="C25" t="n">
-        <v>98.22</v>
-      </c>
-      <c r="D25" t="n">
-        <v>94.09</v>
-      </c>
-      <c r="E25" t="n">
-        <v>83.98999999999999</v>
-      </c>
-      <c r="F25" t="n">
-        <v>19.71</v>
-      </c>
-      <c r="G25" t="n">
-        <v>55.62</v>
-      </c>
-      <c r="H25" t="n">
-        <v>95.01000000000001</v>
-      </c>
-      <c r="I25" t="n">
-        <v>73.97</v>
+      <c r="C29" t="n">
+        <v>755.5384615384615</v>
+      </c>
+      <c r="D29" t="n">
+        <v>723.7692307692308</v>
+      </c>
+      <c r="E29" t="n">
+        <v>646.0769230769231</v>
+      </c>
+      <c r="F29" t="n">
+        <v>151.6153846153846</v>
+      </c>
+      <c r="G29" t="n">
+        <v>427.8461538461539</v>
+      </c>
+      <c r="H29" t="n">
+        <v>730.8461538461539</v>
+      </c>
+      <c r="I29" t="n">
+        <v>569</v>
       </c>
     </row>
   </sheetData>
@@ -3400,7 +3772,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I23"/>
+  <dimension ref="A1:I27"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -3816,67 +4188,67 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>TotalCap-Weight</t>
+          <t>Equal-Weight</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Low</t>
+          <t>DH Ret2</t>
         </is>
       </c>
       <c r="C13" t="n">
-        <v>-0.167</v>
+        <v>0.664</v>
       </c>
       <c r="D13" t="n">
-        <v>-0.163</v>
+        <v>1.184</v>
       </c>
       <c r="E13" t="n">
-        <v>-0.082</v>
+        <v>1.173</v>
       </c>
       <c r="F13" t="n">
-        <v>0.079</v>
+        <v>0.07099999999999999</v>
       </c>
       <c r="G13" t="n">
-        <v>0.123</v>
+        <v>0.489</v>
       </c>
       <c r="H13" t="n">
-        <v>-0.201</v>
+        <v>0.521</v>
       </c>
       <c r="I13" t="n">
-        <v>0.111</v>
+        <v>0.275</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>TotalCap-Weight</t>
+          <t>Equal-Weight</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>DH Ret3</t>
         </is>
       </c>
       <c r="C14" t="n">
-        <v>-0.008999999999999999</v>
+        <v>0.596</v>
       </c>
       <c r="D14" t="n">
-        <v>0.161</v>
+        <v>0.877</v>
       </c>
       <c r="E14" t="n">
-        <v>0.173</v>
+        <v>1.106</v>
       </c>
       <c r="F14" t="n">
-        <v>0.173</v>
+        <v>0.107</v>
       </c>
       <c r="G14" t="n">
-        <v>0.2</v>
+        <v>0.387</v>
       </c>
       <c r="H14" t="n">
-        <v>0.057</v>
+        <v>0.411</v>
       </c>
       <c r="I14" t="n">
-        <v>0.208</v>
+        <v>0.198</v>
       </c>
     </row>
     <row r="15">
@@ -3887,29 +4259,29 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>Low</t>
         </is>
       </c>
       <c r="C15" t="n">
-        <v>0.118</v>
+        <v>-0.167</v>
       </c>
       <c r="D15" t="n">
-        <v>0.193</v>
+        <v>-0.163</v>
       </c>
       <c r="E15" t="n">
-        <v>0.285</v>
+        <v>-0.082</v>
       </c>
       <c r="F15" t="n">
-        <v>0.293</v>
+        <v>0.079</v>
       </c>
       <c r="G15" t="n">
-        <v>0.394</v>
+        <v>0.123</v>
       </c>
       <c r="H15" t="n">
-        <v>0.34</v>
+        <v>-0.201</v>
       </c>
       <c r="I15" t="n">
-        <v>0.3</v>
+        <v>0.111</v>
       </c>
     </row>
     <row r="16">
@@ -3920,29 +4292,29 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>2</t>
         </is>
       </c>
       <c r="C16" t="n">
-        <v>0.308</v>
+        <v>-0.008999999999999999</v>
       </c>
       <c r="D16" t="n">
-        <v>0.294</v>
+        <v>0.161</v>
       </c>
       <c r="E16" t="n">
-        <v>0.3</v>
+        <v>0.173</v>
       </c>
       <c r="F16" t="n">
-        <v>0.378</v>
+        <v>0.173</v>
       </c>
       <c r="G16" t="n">
-        <v>0.447</v>
+        <v>0.2</v>
       </c>
       <c r="H16" t="n">
-        <v>0.323</v>
+        <v>0.057</v>
       </c>
       <c r="I16" t="n">
-        <v>0.345</v>
+        <v>0.208</v>
       </c>
     </row>
     <row r="17">
@@ -3953,29 +4325,29 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>3</t>
         </is>
       </c>
       <c r="C17" t="n">
-        <v>0.381</v>
+        <v>0.118</v>
       </c>
       <c r="D17" t="n">
-        <v>0.344</v>
+        <v>0.193</v>
       </c>
       <c r="E17" t="n">
-        <v>0.389</v>
+        <v>0.285</v>
       </c>
       <c r="F17" t="n">
-        <v>0.465</v>
+        <v>0.293</v>
       </c>
       <c r="G17" t="n">
-        <v>0.595</v>
+        <v>0.394</v>
       </c>
       <c r="H17" t="n">
-        <v>0.446</v>
+        <v>0.34</v>
       </c>
       <c r="I17" t="n">
-        <v>0.487</v>
+        <v>0.3</v>
       </c>
     </row>
     <row r="18">
@@ -3986,29 +4358,29 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>4</t>
         </is>
       </c>
       <c r="C18" t="n">
-        <v>0.465</v>
+        <v>0.308</v>
       </c>
       <c r="D18" t="n">
-        <v>0.49</v>
+        <v>0.294</v>
       </c>
       <c r="E18" t="n">
-        <v>0.399</v>
+        <v>0.3</v>
       </c>
       <c r="F18" t="n">
-        <v>0.55</v>
+        <v>0.378</v>
       </c>
       <c r="G18" t="n">
-        <v>0.54</v>
+        <v>0.447</v>
       </c>
       <c r="H18" t="n">
-        <v>0.595</v>
+        <v>0.323</v>
       </c>
       <c r="I18" t="n">
-        <v>0.555</v>
+        <v>0.345</v>
       </c>
     </row>
     <row r="19">
@@ -4019,29 +4391,29 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>5</t>
         </is>
       </c>
       <c r="C19" t="n">
-        <v>0.535</v>
+        <v>0.381</v>
       </c>
       <c r="D19" t="n">
-        <v>0.523</v>
+        <v>0.344</v>
       </c>
       <c r="E19" t="n">
+        <v>0.389</v>
+      </c>
+      <c r="F19" t="n">
         <v>0.465</v>
       </c>
-      <c r="F19" t="n">
-        <v>0.578</v>
-      </c>
       <c r="G19" t="n">
-        <v>0.506</v>
+        <v>0.595</v>
       </c>
       <c r="H19" t="n">
-        <v>0.62</v>
+        <v>0.446</v>
       </c>
       <c r="I19" t="n">
-        <v>0.595</v>
+        <v>0.487</v>
       </c>
     </row>
     <row r="20">
@@ -4052,29 +4424,29 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>6</t>
         </is>
       </c>
       <c r="C20" t="n">
-        <v>0.709</v>
+        <v>0.465</v>
       </c>
       <c r="D20" t="n">
-        <v>0.5649999999999999</v>
+        <v>0.49</v>
       </c>
       <c r="E20" t="n">
-        <v>0.459</v>
+        <v>0.399</v>
       </c>
       <c r="F20" t="n">
-        <v>0.57</v>
+        <v>0.55</v>
       </c>
       <c r="G20" t="n">
-        <v>0.58</v>
+        <v>0.54</v>
       </c>
       <c r="H20" t="n">
-        <v>0.73</v>
+        <v>0.595</v>
       </c>
       <c r="I20" t="n">
-        <v>0.578</v>
+        <v>0.555</v>
       </c>
     </row>
     <row r="21">
@@ -4085,29 +4457,29 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>7</t>
         </is>
       </c>
       <c r="C21" t="n">
-        <v>0.778</v>
+        <v>0.535</v>
       </c>
       <c r="D21" t="n">
-        <v>0.59</v>
+        <v>0.523</v>
       </c>
       <c r="E21" t="n">
-        <v>0.55</v>
+        <v>0.465</v>
       </c>
       <c r="F21" t="n">
-        <v>0.547</v>
+        <v>0.578</v>
       </c>
       <c r="G21" t="n">
-        <v>0.477</v>
+        <v>0.506</v>
       </c>
       <c r="H21" t="n">
-        <v>0.725</v>
+        <v>0.62</v>
       </c>
       <c r="I21" t="n">
-        <v>0.49</v>
+        <v>0.595</v>
       </c>
     </row>
     <row r="22">
@@ -4118,29 +4490,29 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>8</t>
         </is>
       </c>
       <c r="C22" t="n">
-        <v>0.926</v>
+        <v>0.709</v>
       </c>
       <c r="D22" t="n">
-        <v>0.801</v>
+        <v>0.5649999999999999</v>
       </c>
       <c r="E22" t="n">
-        <v>0.763</v>
+        <v>0.459</v>
       </c>
       <c r="F22" t="n">
-        <v>0.423</v>
+        <v>0.57</v>
       </c>
       <c r="G22" t="n">
-        <v>0.402</v>
+        <v>0.58</v>
       </c>
       <c r="H22" t="n">
-        <v>0.534</v>
+        <v>0.73</v>
       </c>
       <c r="I22" t="n">
-        <v>0.343</v>
+        <v>0.578</v>
       </c>
     </row>
     <row r="23">
@@ -4151,29 +4523,161 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
+          <t>9</t>
+        </is>
+      </c>
+      <c r="C23" t="n">
+        <v>0.778</v>
+      </c>
+      <c r="D23" t="n">
+        <v>0.59</v>
+      </c>
+      <c r="E23" t="n">
+        <v>0.55</v>
+      </c>
+      <c r="F23" t="n">
+        <v>0.547</v>
+      </c>
+      <c r="G23" t="n">
+        <v>0.477</v>
+      </c>
+      <c r="H23" t="n">
+        <v>0.725</v>
+      </c>
+      <c r="I23" t="n">
+        <v>0.49</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>TotalCap-Weight</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="C24" t="n">
+        <v>0.926</v>
+      </c>
+      <c r="D24" t="n">
+        <v>0.801</v>
+      </c>
+      <c r="E24" t="n">
+        <v>0.763</v>
+      </c>
+      <c r="F24" t="n">
+        <v>0.423</v>
+      </c>
+      <c r="G24" t="n">
+        <v>0.402</v>
+      </c>
+      <c r="H24" t="n">
+        <v>0.534</v>
+      </c>
+      <c r="I24" t="n">
+        <v>0.343</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>TotalCap-Weight</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
           <t>H-L</t>
         </is>
       </c>
-      <c r="C23" t="n">
+      <c r="C25" t="n">
         <v>1.521</v>
       </c>
-      <c r="D23" t="n">
+      <c r="D25" t="n">
         <v>1.502</v>
       </c>
-      <c r="E23" t="n">
+      <c r="E25" t="n">
         <v>1.231</v>
       </c>
-      <c r="F23" t="n">
+      <c r="F25" t="n">
         <v>0.174</v>
       </c>
-      <c r="G23" t="n">
+      <c r="G25" t="n">
         <v>0.405</v>
       </c>
-      <c r="H23" t="n">
+      <c r="H25" t="n">
         <v>0.89</v>
       </c>
-      <c r="I23" t="n">
+      <c r="I25" t="n">
         <v>0.351</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>TotalCap-Weight</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>DH Ret2</t>
+        </is>
+      </c>
+      <c r="C26" t="n">
+        <v>0.041</v>
+      </c>
+      <c r="D26" t="n">
+        <v>0.049</v>
+      </c>
+      <c r="E26" t="n">
+        <v>0.204</v>
+      </c>
+      <c r="F26" t="n">
+        <v>0.142</v>
+      </c>
+      <c r="G26" t="n">
+        <v>0.042</v>
+      </c>
+      <c r="H26" t="n">
+        <v>0.105</v>
+      </c>
+      <c r="I26" t="n">
+        <v>0.104</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>TotalCap-Weight</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>DH Ret3</t>
+        </is>
+      </c>
+      <c r="C27" t="n">
+        <v>0.152</v>
+      </c>
+      <c r="D27" t="n">
+        <v>-0.07099999999999999</v>
+      </c>
+      <c r="E27" t="n">
+        <v>0.128</v>
+      </c>
+      <c r="F27" t="n">
+        <v>0.134</v>
+      </c>
+      <c r="G27" t="n">
+        <v>-0.034</v>
+      </c>
+      <c r="H27" t="n">
+        <v>-0.023</v>
+      </c>
+      <c r="I27" t="n">
+        <v>0.226</v>
       </c>
     </row>
   </sheetData>
@@ -4249,25 +4753,25 @@
         </is>
       </c>
       <c r="C2" t="n">
-        <v>90.43000000000001</v>
+        <v>695.6153846153848</v>
       </c>
       <c r="D2" t="n">
-        <v>87.58</v>
+        <v>673.6923076923076</v>
       </c>
       <c r="E2" t="n">
-        <v>76.98</v>
+        <v>592.1538461538462</v>
       </c>
       <c r="F2" t="n">
-        <v>13.02</v>
+        <v>100.1538461538461</v>
       </c>
       <c r="G2" t="n">
-        <v>42.44</v>
+        <v>326.4615384615385</v>
       </c>
       <c r="H2" t="n">
-        <v>84.40000000000001</v>
+        <v>649.2307692307693</v>
       </c>
       <c r="I2" t="n">
-        <v>62.32</v>
+        <v>479.3846153846154</v>
       </c>
     </row>
     <row r="3">
@@ -4282,25 +4786,25 @@
         </is>
       </c>
       <c r="C3" t="n">
-        <v>98.22</v>
+        <v>755.5384615384615</v>
       </c>
       <c r="D3" t="n">
-        <v>94.09</v>
+        <v>723.7692307692308</v>
       </c>
       <c r="E3" t="n">
-        <v>83.98999999999999</v>
+        <v>646.0769230769231</v>
       </c>
       <c r="F3" t="n">
-        <v>19.71</v>
+        <v>151.6153846153846</v>
       </c>
       <c r="G3" t="n">
-        <v>55.62</v>
+        <v>427.8461538461539</v>
       </c>
       <c r="H3" t="n">
-        <v>95.01000000000001</v>
+        <v>730.8461538461539</v>
       </c>
       <c r="I3" t="n">
-        <v>73.97</v>
+        <v>569</v>
       </c>
     </row>
   </sheetData>

</xml_diff>